<commit_message>
Expand all 14 weeks into rigorous bilingual academic notes and language-specific learning materials
</commit_message>
<xml_diff>
--- a/workbooks/Kamu_Diplomasisi_Ogrenme_Atolyesi_TR.xlsx
+++ b/workbooks/Kamu_Diplomasisi_Ogrenme_Atolyesi_TR.xlsx
@@ -12,6 +12,7 @@
     <sheet name="2 Kanıt Çalışması" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="3 Ölçüm Deneyi" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="4 Kavram Rehberi" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="5 Araştırma Tasarımı" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="268">
   <si>
     <t xml:space="preserve">Kamu diplomasisi: ilk adımlar</t>
   </si>
@@ -689,6 +690,144 @@
   </si>
   <si>
     <t xml:space="preserve">Kaynak: Dersin Türkçe notlarındaki kavramsal açıklamalar. Günlük benzetmeler yalnızca öğrenmeyi kolaylaştıran örneklerdir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Araştırma tasarımınızı adım adım kurun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Çözülmüş kurmaca örneği okuyun. 2. Sarı sütuna kendi vakanızı yazın. 3. İddianızı desteklemeyen kanıtı da arayın.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaynak kökeni, belgenin kim tarafından, ne zaman ve hangi amaçla üretildiğini ve size nasıl ulaştığını belirtir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gözlem belgede bulunan şeydir. Yorum, bundan çıkardığınız anlamdır. İkisini ayrı yazmak çıkarımınızı denetlenebilir kılar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Örnek tamamen kurmacadır. ÖRNEK-1 gerçek bir belge kodu değildir. Sarı alanlara öğrenci adı veya kişisel veri yazmayın.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kanıtı sorgulama alanı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Çözülmüş kurmaca örnek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sizin çalışmanız (doldurun)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İddia: Sınadığım cümle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Değişim atölyesi, iki öğretmenin ilk ortak ders planını hazırlamasına katkıda bulundu. Bu, sınanacak iddiadır; henüz sonuç değildir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaynak kökeni: Belgeyi kim üretti?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ÖRNEK-1: Katılımcı A’nın katılımcı B’ye atölye sonrasında yazdığı varsayılan özel mektup. Üretici, alıcı, tarih, amaç ve saklandığı yer gerçek araştırmada ayrıca doğrulanır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gözlem: Belgede tam olarak ne var?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Varsayılan mektup, ortak bir ders taslağından söz eder. Bu gözlem, mektubun içeriğine ilişkindir; taslağın uygulandığını göstermez.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yorum: Bu gözlemden ne çıkarıyorum?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atölye sonrasında iletişimin sürmüş olmasıyla uyumludur. Atölyenin tek neden olduğu veya ilişkinin kalıcı olduğu sonucuna yetmez.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rakip açıklama: Başka neden olabilir mi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Öğretmenler önceden tanışıyor veya başka bir proje için zaten işbirliği planlıyor olabilir. Atölye öncesi yazışmalar bu açıklamayı sınayabilir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sınırlılık: Kanıtımın sınırı nedir?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tek bir öz bildirime dayanır. Yazışmanın seçilerek korunması, olumlu anlatım ve karşı tarafın sessizliği sonucu çarpıtabilir. İletişim, politika değişikliği anlamına gelmez.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sonraki kanıt: Neyi kontrol edeceğim?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atölye öncesi kayıtları, ikinci katılımcının anlatısını ve tarihli ortak taslağı karşılaştırırım. Çelişki bulursam iddiayı daraltırım; aynı kaynağın tekrarını bağımsız doğrulama saymam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Şimdi tasarım kararları: Her satır bir araştırma tercihini açık eder. Veri yoksa sonuç uydurmak yerine hangi veriyi arayacağınızı yazın.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasarım kararı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Örnekte nasıl uygulanır?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benim araştırma planım</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Araştırma sorusu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atölye, belirli iki öğretmenin ilk ortak ders taslağını hazırlamasına hangi süreçle katkıda bulundu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İnceleme birimi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bir öğretmen çifti ve onun ortak çalışma süreci. Kişi, etkinlik ve ülke düzeyindeki iddiaları birbirine karıştırmam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaman ve kapsam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Varsayımsal plan: atölyeden önceki ve sonraki üç ay. Bu sınırın dışındaki olayları ancak gerekçesini belirterek eklerim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beklenen mekanizma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atölyede temas kurulması, ortak bir konu seçilmesi ve birlikte taslak hazırlanması. Her adım için ayrı bir iz ararım.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gösterge ve tanımı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarih ve ortak katkı izi bulunan ders taslağı. Katılım listesi yalnız katılımı gösterir; ortak üretimin yerine geçmez.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vaka seçimi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yalnız başarı anlatılarını seçmem. Devam etmeyen temasları da arar, hangi kişilerin veya belgelerin neden dışarıda kaldığını kaydederim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karşılaştırma ve karşı olgu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atölye öncesindeki işbirliğini ve uygun benzer katılmayan kişileri araştırırım. Grupların başlangıçta farklı olabileceğini açıklarım; benzerliği otomatik varsaymam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etik ve veri yönetimi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gönüllü katılım, uygun izin, kişisel bilgilerin azaltılması ve güvenli saklama planı kurarım. Öğrenci verilerini bu çalışma kitabına kopyalamam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaynak gösterme ve denetim izi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yazar, tarih, başlık, koleksiyon veya yayın, kayıt/sayfa ve erişim bilgisini kaydederim. Çeviri, eksik belge ve değişen yorum için kısa bir işlem günlüğü tutarım.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teslim öncesi: İddia, gözlem, yorum ve sınır ayrı mı? En güçlü rakip açıklamayı sınamak için hangi kanıt gerekiyor?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ders dayanağı: 6. hafta değişimler, 14. hafta kanıt ve değerlendirme. Kurmaca örnek herhangi bir tarihsel sonuca kanıt oluşturmaz.</t>
   </si>
 </sst>
 </file>
@@ -1348,11 +1487,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="96920239"/>
-        <c:axId val="79127438"/>
+        <c:axId val="73527653"/>
+        <c:axId val="48016607"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="96920239"/>
+        <c:axId val="73527653"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1397,7 +1536,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79127438"/>
+        <c:crossAx val="48016607"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1405,7 +1544,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79127438"/>
+        <c:axId val="48016607"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1450,7 +1589,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96920239"/>
+        <c:crossAx val="73527653"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4172,4 +4311,380 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF801C35"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="59.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="2.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="31" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+      <c r="B9" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+      <c r="B10" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+      <c r="B11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="D11" s="12"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+      <c r="B12" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D12" s="12"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+      <c r="B13" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="D13" s="12"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1"/>
+      <c r="B14" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="D14" s="12"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1"/>
+      <c r="B15" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="D15" s="12"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1"/>
+      <c r="B16" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="D16" s="16"/>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1"/>
+      <c r="B20" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1"/>
+      <c r="B21" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="D21" s="8"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1"/>
+      <c r="B22" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="D22" s="12"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1"/>
+      <c r="B23" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="D23" s="12"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1"/>
+      <c r="B24" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="D24" s="12"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1"/>
+      <c r="B25" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="D25" s="12"/>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1"/>
+      <c r="B26" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="D26" s="12"/>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1"/>
+      <c r="B27" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="D27" s="12"/>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1"/>
+      <c r="B28" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="D28" s="12"/>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1"/>
+      <c r="B29" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="D29" s="16"/>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1"/>
+      <c r="B34" s="25" t="str">
+        <f aca="false">HYPERLINK("https://mayhewforever.github.io/kamudiplomasisi/notes/Hafta_06_Ders_Notu_TR.html","6. hafta: değişimler")</f>
+        <v>6. hafta: değişimler</v>
+      </c>
+      <c r="C34" s="25" t="str">
+        <f aca="false">HYPERLINK("https://mayhewforever.github.io/kamudiplomasisi/notes/Hafta_14_Ders_Notu_TR.html","14. hafta: ölçüm")</f>
+        <v>14. hafta: ölçüm</v>
+      </c>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+    </row>
+    <row r="35" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+    </row>
+    <row r="36" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Revise all bilingual course notes and exercises into an academic register
Formalise English and Turkish explanations, definitions, cases and model answers while retaining historical qualifications and accessible structure. Regenerate 28 reading pages and PDFs, update both Excel workbooks, and correct PDF callout/reference pagination.
</commit_message>
<xml_diff>
--- a/workbooks/Kamu_Diplomasisi_Ogrenme_Atolyesi_TR.xlsx
+++ b/workbooks/Kamu_Diplomasisi_Ogrenme_Atolyesi_TR.xlsx
@@ -24,24 +24,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="268">
-  <si>
-    <t xml:space="preserve">Kamu diplomasisi: ilk adımlar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Bu hafta hangi konuyu işliyorsanız o satırı bulun. “Ders notunu aç” bağlantısına tıklayın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. “Küçük görev” sütununu uygulayın. “Yazacağınız sonuç” kadar kısa bir cevap hazırlayın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Sarı durum hücresinden seçin. Sonra 2. sayfadaki örneği okuyup kendi kanıt satırınızı doldurun.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gündelik benzetme: Bir afişi görmek, afişte önerilen ürünü beğenmek veya satın almakla aynı şey değildir.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excel ipucu: Sarı hücreye tıklayın, yazın ve Enter’a basın. Diğer sayfalara alttaki sekmelerden geçin.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="267">
+  <si>
+    <t xml:space="preserve">Kamu diplomasisi: haftalık çalışma rehberi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. İlgili haftanın satırını belirleyiniz. “Ders notunu aç” bağlantısından haftalık okuma metnine ulaşınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. “Uygulama” sütunundaki çalışmayı tamamlayınız. “Beklenen çıktı” sütununda belirtilen kapsamda kısa bir yanıt hazırlayınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Sarı hücrede çalışma durumunu seçiniz. Ardından 2. sayfadaki örneği inceleyerek kanıt tablosunda bir satır doldurunuz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Açıklayıcı benzetme: Bir afişle karşılaşılması, tanıtılan ürünün beğenildiğini veya satın alındığını tek başına göstermez.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Çalışma kitabının kullanımı: Sarı hücreyi seçip veriyi giriniz ve Enter’a basınız. Sayfalar arasında alt sekmelerden geçiş yapınız.</t>
   </si>
   <si>
     <t xml:space="preserve">Hafta</t>
@@ -50,25 +50,25 @@
     <t xml:space="preserve">Konu</t>
   </si>
   <si>
-    <t xml:space="preserve">Küçük görev</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yazacağınız sonuç</t>
+    <t xml:space="preserve">Uygulama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beklenen çıktı</t>
   </si>
   <si>
     <t xml:space="preserve">Ders notu</t>
   </si>
   <si>
-    <t xml:space="preserve">Durum (siz seçin)</t>
+    <t xml:space="preserve">Çalışma durumu</t>
   </si>
   <si>
     <t xml:space="preserve">Güç türlerini ayırmak</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir burs örneği seçin. Para, çekicilik ve beklenen sonucu ayrı yazın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Üç cümle: kaynak ne, araç ne, sonuç için hangi kanıt eksik?</t>
+    <t xml:space="preserve">Bir burs örneği seçiniz. Finansman kaynağını, çekiciliği ve beklenen sonucu ayrı ayrı belirtiniz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Üç cümlede kaynağı, aracı ve sonucu değerlendirmek için gereken ek kanıtı belirtiniz.</t>
   </si>
   <si>
     <t xml:space="preserve">Başlamadım</t>
@@ -77,16 +77,16 @@
     <t xml:space="preserve">Franklin ve Fransa</t>
   </si>
   <si>
-    <t xml:space="preserve">Franklin’in bir bilim veya toplum ağı temasını seçin. Teması, ittifak kararından ayırın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">İki neden: temasın katkısı ne olabilir, kararın başka nedeni ne olabilir?</t>
+    <t xml:space="preserve">Franklin’in bilimsel veya toplumsal ağlardaki bir temasını seçiniz. Bu teması ittifak kararından analitik olarak ayırınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temasın olası katkısına ve kararı açıklayabilecek başka bir nedene ilişkin iki açıklama.</t>
   </si>
   <si>
     <t xml:space="preserve">Birlik ve Avrupa</t>
   </si>
   <si>
-    <t xml:space="preserve">Birlik yönetiminin bir anlatısını bulun. Avrupa’daki hangi kitleye seslendiğini yazın.</t>
+    <t xml:space="preserve">Birlik yönetiminin kullandığı bir anlatıyı belirleyiniz. Avrupa’da yöneldiği hedef kitleyi açıklayınız.</t>
   </si>
   <si>
     <t xml:space="preserve">Bir mesaj, bir kitle, mesajın nasıl karşılandığını gösterecek bir belge türü.</t>
@@ -95,34 +95,34 @@
     <t xml:space="preserve">Konfederasyon ve pamuk</t>
   </si>
   <si>
-    <t xml:space="preserve">Pamuk kaynağının neden otomatik siyasi destek üretmediğini açıklayın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bir kaynak, bir beklenen sonuç, zinciri bozabilecek iki koşul.</t>
+    <t xml:space="preserve">Pamuk kaynağının neden kendiliğinden siyasi desteğe dönüşmediğini açıklayınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bir kaynak, bir beklenen sonuç ve öngörülen süreci kesintiye uğratabilecek iki koşul.</t>
   </si>
   <si>
     <t xml:space="preserve">Küba ve insani yardım</t>
   </si>
   <si>
-    <t xml:space="preserve">Yardım faaliyeti ile yardımın medyada anlatılmasını ayrı düşünün.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faaliyet için bir kanıt, habercilik için bir kanıt, etki için bir eksik kanıt.</t>
+    <t xml:space="preserve">Yardım faaliyetini, bu faaliyetin medyadaki temsilinden ayırarak inceleyiniz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faaliyete ve haberciliğe ilişkin birer kanıt ile etkiyi değerlendirmek için gereken ek kanıt.</t>
   </si>
   <si>
     <t xml:space="preserve">Eğitim değişimleri</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir öğrenci değişim programında ev sahibi ile katılımcının ne öğrendiğini yazın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Katılım sayısının yanında izleyeceğiniz bir ilişki göstergesi.</t>
+    <t xml:space="preserve">Bir öğrenci değişim programında ev sahibi ile katılımcının öğrenme deneyimlerini ayrı ayrı açıklayınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Katılım sayısına ek olarak izlenebilecek bir ilişki göstergesi.</t>
   </si>
   <si>
     <t xml:space="preserve">CPI ve iletişim ağı</t>
   </si>
   <si>
-    <t xml:space="preserve">Kamuoyu Bilgilendirme Komitesini (CPI) merkez, aracı ve kitle olarak üç kutuya ayırın.</t>
+    <t xml:space="preserve">Kamuoyu Bilgilendirme Komitesinin (CPI) iletişim ağını merkez, aracı ve kitle başlıklarıyla üç kutuda gösteriniz.</t>
   </si>
   <si>
     <t xml:space="preserve">Bir afişin üretilmesi ile bir kişinin ikna olması arasındaki eksik adım.</t>
@@ -131,7 +131,7 @@
     <t xml:space="preserve">Propaganda ve etik</t>
   </si>
   <si>
-    <t xml:space="preserve">Doğru bilgiler içeren ama kaynağı gizli bir mesajı değerlendirin.</t>
+    <t xml:space="preserve">Doğru bilgiler içeren ancak kaynağı açıklanmayan bir mesajı değerlendiriniz.</t>
   </si>
   <si>
     <t xml:space="preserve">Kaynak, eksik bağlam ve düzeltme yolu hakkında üç soru.</t>
@@ -140,7 +140,7 @@
     <t xml:space="preserve">Vakıflar ve özel ağlar</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir vakıf veya üniversite örneği seçin. Kimin finansman verdiğini ve kararı kimin aldığını ayırın.</t>
+    <t xml:space="preserve">Bir vakıf veya üniversite örneği seçiniz. Finansman sağlayan aktörlerle karar alan aktörleri ayırınız.</t>
   </si>
   <si>
     <t xml:space="preserve">İki aktör ve birbirlerinden bağımsız olabilecekleri bir nokta.</t>
@@ -149,25 +149,25 @@
     <t xml:space="preserve">Savaş dönemi kurumları</t>
   </si>
   <si>
-    <t xml:space="preserve">Notta tanıtılan üç kurumu amaç, hedef insanlar ve kullanılan araç başlıklarında karşılaştırın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Üç kısa satır. Aynı aracı kullanmanın neden aynı görev olmadığını ekleyin.</t>
+    <t xml:space="preserve">Ders notundaki üç kurumu amaç, hedef kamu ve kullanılan araç bakımından karşılaştırınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Üç kısa karşılaştırma satırı. Aynı aracın kullanılmasının neden aynı kurumsal göreve işaret etmediğini açıklayınız.</t>
   </si>
   <si>
     <t xml:space="preserve">Radyo, sinema ve basın</t>
   </si>
   <si>
-    <t xml:space="preserve">Aynı mesajın radyo, film ve gazetede nasıl farklı karşılanabileceğini düşünün.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Üç mecra için birer avantaj ve birer sınır.</t>
+    <t xml:space="preserve">Aynı mesajın radyo, sinema ve gazetede nasıl farklı alımlanabileceğini değerlendiriniz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Üç mecranın her biri için bir avantaj ve bir sınırlılık.</t>
   </si>
   <si>
     <t xml:space="preserve">Smith–Mundt ve kurumlar</t>
   </si>
   <si>
-    <t xml:space="preserve">Yasal yetki, uygulama kapasitesi ve sonuç için ayrı kanıtlar belirleyin.</t>
+    <t xml:space="preserve">Yasal yetki, uygulama kapasitesi ve sonuç için ayrı kanıtlar belirleyiniz.</t>
   </si>
   <si>
     <t xml:space="preserve">Bir yasanın neyi mümkün kıldığı ve neyi tek başına kanıtlamadığı.</t>
@@ -176,7 +176,7 @@
     <t xml:space="preserve">Ülkeler arası karşılaştırma</t>
   </si>
   <si>
-    <t xml:space="preserve">İki kültür kurumu veya yayıncıyı aynı üç soruyla karşılaştırın: kim yönetir, kime ulaşır, nasıl geri bildirim alır?</t>
+    <t xml:space="preserve">İki kültür kurumunu veya yayıncıyı yönetim, hedef kitle ve geri bildirim süreçleri bakımından karşılaştırınız.</t>
   </si>
   <si>
     <t xml:space="preserve">İki satırlık karşılaştırma ve sonucu etkileyebilecek bir bağlam farkı.</t>
@@ -185,31 +185,31 @@
     <t xml:space="preserve">Etkiyi değerlendirmek</t>
   </si>
   <si>
-    <t xml:space="preserve">3. sayfadaki sarı sayılardan birini değiştirin. Erişim ve destek değişimini ayrı okuyun.</t>
+    <t xml:space="preserve">3. sayfadaki sarı girdi hücrelerinden birini değiştiriniz. Erişimi ve destek değişimini ayrı ayrı yorumlayınız.</t>
   </si>
   <si>
     <t xml:space="preserve">Dört cümle: amaç, gözlem, başka açıklama ve ek kanıt ihtiyacı.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kendi cümleniz için şablon: “Bu kaynak … gösteriyor. … sonucuna ulaşmak için ayrıca … gerekir.”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Örnek: “Afiş, mesajın üretildiğini gösteriyor. İkna sonucuna ulaşmak için kitlenin tepkisini de bilmem gerekir.”</t>
+    <t xml:space="preserve">Analitik ifade şablonu: “Bu kaynak … göstermektedir. … sonucuna ulaşmak için ayrıca … kanıtı gereklidir.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Örnek: “Afiş, mesajın üretildiğini göstermektedir. İkna sonucuna ulaşmak için kitlenin tepkisine ilişkin kanıt da gereklidir.”</t>
   </si>
   <si>
     <t xml:space="preserve">Kaynak: Bu sitedeki 14 haftalık Türkçe ders notu. Bağlantılar yukarıdaki ilgili hafta satırındadır.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir iddiayı kanıtla nasıl sınarım?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. “Ne söylüyorum?” sorusuna tek cümle yazın. 2. Elinizdeki belgeyi belirtin. 3. Belgenin sınırını yazın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kanıt = iddiayı destekleyen iz. “Kanıt matrisi”, bu izleri aynı sorularla karşılaştırdığınız aşağıdaki tablodur.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gündelik örnek: Kafenin ilanını görmek, oradan kahve satın aldığınızı kanıtlamaz. Aradaki adımı ayrı gösterin.</t>
+    <t xml:space="preserve">İddiaların kanıt temelinde sınanması</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. İddiayı tek cümleyle ifade ediniz. 2. İncelenen belgeyi belirtiniz. 3. Belgenin kanıtlama sınırlarını açıklayınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kanıt, bir iddiayı destekleyen izdir. Aşağıdaki kanıt matrisi, bu izlerin ortak sorular temelinde karşılaştırılmasını sağlar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Açıklayıcı örnek: Kafe ilanıyla karşılaşılması, kahve satın alındığını göstermez. İki olay arasındaki eksik adımı belirleyiniz.</t>
   </si>
   <si>
     <t xml:space="preserve">Çözülmüş örnekler: Aşağıdaki belge türleri öğretim içindir. Bunlar bulunmuş gerçek arşiv belgeleri değildir.</t>
@@ -218,19 +218,19 @@
     <t xml:space="preserve">Örnek</t>
   </si>
   <si>
-    <t xml:space="preserve">Ne söylüyorum? (iddia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neye bakıyorum? (belge türü)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belge neyi gösterebilir?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tek başına neyi göstermez?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Başka ne açıklayabilir?</t>
+    <t xml:space="preserve">Sınanan iddia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İncelenen belge türü</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgenin gösterebileceği husus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tek başına gösteremeyeceği husus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olası rakip açıklama</t>
   </si>
   <si>
     <t xml:space="preserve">Ders bağlantısı</t>
@@ -290,22 +290,19 @@
     <t xml:space="preserve">Yerel yorumlar ve mevcut görüşler farklı olabilir.</t>
   </si>
   <si>
-    <t xml:space="preserve">Şimdi siz: Bir ders notundan olay seçin. Sarı satırı doldurun. Belgeyi görmediyseniz “aranacak belge” yazın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vakam / haftam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ne söylüyorum?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belgem / arayacağım belge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bundan ne öğrenirim?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neyi hâlâ bilmiyorum?</t>
+    <t xml:space="preserve">Uygulama: Ders notundan bir vaka seçerek sarı satırı doldurunuz. İncelenmemiş belgeleri “aranacak belge” olarak belirtiniz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vaka / hafta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belge / aranacak belge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgeden çıkarılabilecek bilgi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yanıtlanmamış sorular</t>
   </si>
   <si>
     <t xml:space="preserve">Başka açıklama</t>
@@ -326,28 +323,28 @@
     <t xml:space="preserve">Uygulama 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Kendinizi kontrol edin: “Belge var” mı dedim, “etki var” mı dedim? İkincisini yazdıysam aradaki yolu gösterebildim mi?</t>
+    <t xml:space="preserve">Değerlendirme: Belgenin varlığı ile etkiye ilişkin iddia ayrılmış mıdır? Etki iddiası varsa bağlantıyı kuran adımlar gösterilmiş midir?</t>
   </si>
   <si>
     <t xml:space="preserve">Örneklere temel: 6. hafta eğitim değişimi, 7. hafta CPI, 11. hafta medya. İlgili ders notları örnek satırlarında bağlıdır.</t>
   </si>
   <si>
-    <t xml:space="preserve">Erişim ile destek değişimini ayırın</t>
+    <t xml:space="preserve">Erişim ve destek değişiminin karşılaştırılması</t>
   </si>
   <si>
     <t xml:space="preserve">Tamamen varsayımsal veri: A ve B hayalî kampanyalardır. Sayılar gerçek kişi, öğrenci veya tarihsel olay verisi değildir.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Sarı hücrelere bakın. 2. Önce aşağıdaki çözülmüş örneği okuyun. 3. D10’u 600 yapıp sonuçları izleyin.</t>
+    <t xml:space="preserve">1. Sarı girdi hücrelerini inceleyiniz. 2. Aşağıdaki çözülmüş örneği okuyunuz. 3. D10’a 600 girerek sonuçlardaki değişimi gözlemleyiniz.</t>
   </si>
   <si>
     <t xml:space="preserve">Başlangıç örneğinde, her kampanyada ulaşılanlardan seçilmiş aynı 100 kişiye önce ve sonra aynı destek sorusu soruldu.</t>
   </si>
   <si>
-    <t xml:space="preserve">“Destek” = soruya olumlu yanıt. İkna için daha güçlü kanıt gerekir. Kontrol grubu olmayan bu gözlem neden-sonuç kanıtlamaz.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kontrol grubu = kampanyayı almayan, karşılaştırma için izlenen benzer kişiler. Bu örnekte böyle bir grup yok.</t>
+    <t xml:space="preserve">“Destek”, soruya verilen olumlu yanıttır. İkna iddiası daha güçlü kanıt gerektirir. Kontrol grubu bulunmayan bu gözlem nedenselliği kanıtlamaz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrol grubu, kampanyaya maruz kalmayan ve karşılaştırma amacıyla izlenen benzer kişilerden oluşur. Bu örnekte kontrol grubu bulunmamaktadır.</t>
   </si>
   <si>
     <t xml:space="preserve">Kampanya</t>
@@ -392,10 +389,10 @@
     <t xml:space="preserve">Değişim (yüzde puan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hesap nasıl yapılır?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sonucu nasıl okurum?</t>
+    <t xml:space="preserve">Hesaplama yöntemi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sonucun yorumu</t>
   </si>
   <si>
     <t xml:space="preserve">Erişim = ulaşan ÷ hedef.</t>
@@ -407,22 +404,22 @@
     <t xml:space="preserve">Çözülmüş başlangıç örneği: A’da 800 ÷ 1.000 = %80 erişim. Destek %40’tan %44’e çıkar: 4 yüzde puan.</t>
   </si>
   <si>
-    <t xml:space="preserve">B’de başlangıç erişimi daha düşüktür (%40). Destek artışı daha büyüktür (15 yüzde puan). Görülmek ile ikna ayrı sorulardır.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alıştırma 1: D10’u 800’den 600’e değiştirin. Erişim %60 olur. Destek değişimi neden aynı kalır?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alıştırma 2: G10’u 44’ten 60’a değiştirin. Destek %60 olur ve artış 20 yüzde puana çıkar. Hangi veri değişti?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alıştırma 3: E10’u boş bırakın. Sonucun kaybolması neden %0 görünmesinden daha dürüsttür? Sonra 100 yazın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alıştırma 4: “B daha çok ikna etti” demeden önce ne öğrenmelisiniz? Başlangıç farkları ve başka olayları düşünün.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cevabınız</t>
+    <t xml:space="preserve">B’de başlangıç erişimi daha düşük (%40), destek artışı daha yüksektir (15 yüzde puan). Maruz kalma ile ikna ayrı ayrı değerlendirilmelidir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alıştırma 1: D10’u 800’den 600’e değiştiriniz. Erişim %60 olur. Destek değişiminin neden sabit kaldığını açıklayınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alıştırma 2: G10’u 44’ten 60’a değiştiriniz. Destek %60, artış 20 yüzde puan olur. Değişen girdiyi belirleyiniz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alıştırma 3: E10’u boş bırakınız. Eksik veri için sonucun boş kalmasının neden %0 gösterilmesinden uygun olduğunu açıklayınız. Ardından 100 giriniz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alıştırma 4: B’nin daha fazla ikna sağladığı iddiası için gereken ek kanıtı belirtiniz. Başlangıç farklarını ve diğer olayları değerlendiriniz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yanıt</t>
   </si>
   <si>
     <t xml:space="preserve">Erişim neyi ölçer?</t>
@@ -437,16 +434,16 @@
     <t xml:space="preserve">Hangi ek veri gerekir?</t>
   </si>
   <si>
-    <t xml:space="preserve">Kararımın sınırı</t>
+    <t xml:space="preserve">Sonucun sınırlılığı</t>
   </si>
   <si>
     <t xml:space="preserve">Bir cümlelik sonuç</t>
   </si>
   <si>
-    <t xml:space="preserve">Benim açıklamam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formülü görmek için C16’ya tıklayın. Üstteki formül çubuğunda D10/C10, yani “ulaşan kişi / hedef kişi” görünür.</t>
+    <t xml:space="preserve">Analitik açıklama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formülü incelemek için C16’yı seçiniz. Formül çubuğundaki D10/C10, “ulaşılan kişi sayısı / hedef kişi sayısı” oranını ifade eder.</t>
   </si>
   <si>
     <t xml:space="preserve">Yüzde puan: %40 ile %44 arasındaki fark 4 puandır. Göreli yüzde artışı ise %10’dur. Bunlar farklı ölçülerdir.</t>
@@ -455,31 +452,31 @@
     <t xml:space="preserve">Kaynak: Bu sayfadaki sayılar öğretim amacıyla kuruldu. Kavramlar dersin 1. ve 14. hafta notlarına dayanır.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kavramları günlük dille okuyun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Bilmediğiniz sözcüğü bulun. 2. Günlük örneği okuyun. 3. Son sütundaki soruyu seçtiğiniz ders vakasına uygulayın.</t>
+    <t xml:space="preserve">Temel kavramlar ve açıklayıcı benzetmeler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. İncelenecek kavramı belirleyiniz. 2. Açıklayıcı örneği okuyunuz. 3. Son sütundaki soruyu seçilen ders vakasına uygulayınız.</t>
   </si>
   <si>
     <t xml:space="preserve">Kavram</t>
   </si>
   <si>
-    <t xml:space="preserve">Kısaca anlamı</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Günlük benzetme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kendinize sorun</t>
+    <t xml:space="preserve">Kısa tanım</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Açıklayıcı benzetme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analitik soru</t>
   </si>
   <si>
     <t xml:space="preserve">Aktör</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir şey yapmaya çalışan kişi veya kuruluş.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kafe sahibi bir ilan hazırlatıyor.</t>
+    <t xml:space="preserve">Belirli bir amacı gerçekleştirmeye çalışan kişi veya kuruluş.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bir kafe sahibinin ilan hazırlatması.</t>
   </si>
   <si>
     <t xml:space="preserve">Kim, neyi değiştirmeye çalışıyor?</t>
@@ -494,7 +491,7 @@
     <t xml:space="preserve">Kafenin çevresindeki öğrenciler.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hangi insanlar? Hepsini aynı mı sayıyorum?</t>
+    <t xml:space="preserve">Hangi gruplar incelenmektedir? Aralarındaki farklılıklar dikkate alınmış mıdır?</t>
   </si>
   <si>
     <t xml:space="preserve">Kaynak</t>
@@ -512,7 +509,7 @@
     <t xml:space="preserve">Araç</t>
   </si>
   <si>
-    <t xml:space="preserve">Kaynağın insanlarla temas etme biçimi.</t>
+    <t xml:space="preserve">Bir kaynağın insanlarla etkileşim kurmak için kullanılma biçimi.</t>
   </si>
   <si>
     <t xml:space="preserve">İlan, tanıtım etkinliği veya davet.</t>
@@ -524,19 +521,19 @@
     <t xml:space="preserve">Mekanizma</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir şeyin başka bir şeyi nasıl değiştirebileceğini anlatan yol.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Güvenilir bir tavsiye, deneme isteği doğuruyor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aradaki adım ne? Bu adımı gözleyebilir miyim?</t>
+    <t xml:space="preserve">Bir etkenin başka bir etkeni nasıl değiştirebileceğini açıklayan süreç.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Güvenilir bir tavsiyenin deneme isteğini artırması.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ara aşama nedir? Bu aşama gözlemlenebilir mi?</t>
   </si>
   <si>
     <t xml:space="preserve">Erişim</t>
   </si>
   <si>
-    <t xml:space="preserve">İnsanların içerikle karşılaşması. Tanımını ve sayım yöntemini belirtin.</t>
+    <t xml:space="preserve">İnsanların içerikle karşılaşması. Tanımın ve sayım yönteminin belirtilmesi gerekir.</t>
   </si>
   <si>
     <t xml:space="preserve">Kaç kişi ilanı gerçekten gördü?</t>
@@ -551,10 +548,10 @@
     <t xml:space="preserve">İnsanların mesajı nasıl anladığı ve değerlendirdiği.</t>
   </si>
   <si>
-    <t xml:space="preserve">Aynı ilanı biri faydalı, biri itici bulur.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kitle ne anlam çıkardı? Kendi sesini duyuyor muyum?</t>
+    <t xml:space="preserve">Aynı ilanın bir kişi tarafından yararlı, diğeri tarafından itici bulunması.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kitle mesajı nasıl yorumlamıştır? Kitlenin kendi ifadelerine ilişkin kanıt var mıdır?</t>
   </si>
   <si>
     <t xml:space="preserve">Tutum ve davranış</t>
@@ -566,7 +563,7 @@
     <t xml:space="preserve">Kafeyi sevmek tutum, alışveriş yapmak davranıştır.</t>
   </si>
   <si>
-    <t xml:space="preserve">Düşünce mi, eylem mi ölçüyorum?</t>
+    <t xml:space="preserve">Ölçülen unsur bir değerlendirme mi, gözlenebilir eylem mi?</t>
   </si>
   <si>
     <t xml:space="preserve">Sert güç</t>
@@ -590,7 +587,7 @@
     <t xml:space="preserve">Birini, iyi örnek olduğu için izlemek.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hayranlığı politika desteğiyle karıştırıyor muyum?</t>
+    <t xml:space="preserve">Hayranlık ile politika desteği analitik olarak ayrılmış mıdır?</t>
   </si>
   <si>
     <t xml:space="preserve">Kamu diplomasisi</t>
@@ -626,7 +623,7 @@
     <t xml:space="preserve">Yanlışını açıkça düzelten bir konuşmacı.</t>
   </si>
   <si>
-    <t xml:space="preserve">İnanma nedenini nasıl biliyorum?</t>
+    <t xml:space="preserve">Kaynağa duyulan güvenin nedenleri hangi kanıta dayanmaktadır?</t>
   </si>
   <si>
     <t xml:space="preserve">Karşılıklılık</t>
@@ -674,7 +671,7 @@
     <t xml:space="preserve">800 ulaşan / 1.000 hedef = %80.</t>
   </si>
   <si>
-    <t xml:space="preserve">Aynı kitle ve dönemden sayıları mı bölüyorum?</t>
+    <t xml:space="preserve">Pay ve payda aynı kitleye ve döneme mi ilişkindir?</t>
   </si>
   <si>
     <t xml:space="preserve">Yüzde puan</t>
@@ -686,25 +683,25 @@
     <t xml:space="preserve">%40’tan %44’e geçiş 4 yüzde puandır.</t>
   </si>
   <si>
-    <t xml:space="preserve">Yüzde artışıyla karıştırıyor muyum?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaynak: Dersin Türkçe notlarındaki kavramsal açıklamalar. Günlük benzetmeler yalnızca öğrenmeyi kolaylaştıran örneklerdir.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Araştırma tasarımınızı adım adım kurun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Çözülmüş kurmaca örneği okuyun. 2. Sarı sütuna kendi vakanızı yazın. 3. İddianızı desteklemeyen kanıtı da arayın.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaynak kökeni, belgenin kim tarafından, ne zaman ve hangi amaçla üretildiğini ve size nasıl ulaştığını belirtir.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gözlem belgede bulunan şeydir. Yorum, bundan çıkardığınız anlamdır. İkisini ayrı yazmak çıkarımınızı denetlenebilir kılar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Örnek tamamen kurmacadır. ÖRNEK-1 gerçek bir belge kodu değildir. Sarı alanlara öğrenci adı veya kişisel veri yazmayın.</t>
+    <t xml:space="preserve">Yüzde puan ile göreli yüzde artışı ayrılmış mıdır?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaynak: Dersin Türkçe notlarındaki kavramsal açıklamalar. Açıklayıcı benzetmeler yalnızca öğrenmeyi kolaylaştıran örneklerdir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Araştırma tasarımının aşamaları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Çözülmüş kurmaca örneği inceleyiniz. 2. Seçilen vakayı sarı sütunda açıklayınız. 3. İddiayla çelişebilecek kanıtları da araştırınız.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaynak kökeni, belgenin üreticisini, tarihini, amacını ve araştırmacıya hangi yolla ulaştığını belirtir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gözlem, belgede yer alan bilgidir. Yorum, bu bilgiden yapılan çıkarımdır. İkisinin ayrı belirtilmesi, çıkarımın denetlenmesini sağlar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Örnek tamamen kurmacadır. ÖRNEK-1 gerçek bir belge kodu değildir. Sarı alanlara öğrenci adı veya kişisel veri girmeyiniz.</t>
   </si>
   <si>
     <t xml:space="preserve">Kanıtı sorgulama alanı</t>
@@ -713,10 +710,10 @@
     <t xml:space="preserve">Çözülmüş kurmaca örnek</t>
   </si>
   <si>
-    <t xml:space="preserve">Sizin çalışmanız (doldurun)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">İddia: Sınadığım cümle</t>
+    <t xml:space="preserve">Araştırma uygulaması</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İddia: Sınanacak önerme</t>
   </si>
   <si>
     <t xml:space="preserve">Değişim atölyesi, iki öğretmenin ilk ortak ders planını hazırlamasına katkıda bulundu. Bu, sınanacak iddiadır; henüz sonuç değildir.</t>
@@ -728,13 +725,13 @@
     <t xml:space="preserve">ÖRNEK-1: Katılımcı A’nın katılımcı B’ye atölye sonrasında yazdığı varsayılan özel mektup. Üretici, alıcı, tarih, amaç ve saklandığı yer gerçek araştırmada ayrıca doğrulanır.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gözlem: Belgede tam olarak ne var?</t>
+    <t xml:space="preserve">Gözlem: Belgenin içerdiği bilgi</t>
   </si>
   <si>
     <t xml:space="preserve">Varsayılan mektup, ortak bir ders taslağından söz eder. Bu gözlem, mektubun içeriğine ilişkindir; taslağın uygulandığını göstermez.</t>
   </si>
   <si>
-    <t xml:space="preserve">Yorum: Bu gözlemden ne çıkarıyorum?</t>
+    <t xml:space="preserve">Yorum: Gözlemden yapılan çıkarım</t>
   </si>
   <si>
     <t xml:space="preserve">Atölye sonrasında iletişimin sürmüş olmasıyla uyumludur. Atölyenin tek neden olduğu veya ilişkinin kalıcı olduğu sonucuna yetmez.</t>
@@ -746,28 +743,28 @@
     <t xml:space="preserve">Öğretmenler önceden tanışıyor veya başka bir proje için zaten işbirliği planlıyor olabilir. Atölye öncesi yazışmalar bu açıklamayı sınayabilir.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sınırlılık: Kanıtımın sınırı nedir?</t>
+    <t xml:space="preserve">Sınırlılık: Kanıtın açıklama sınırı</t>
   </si>
   <si>
     <t xml:space="preserve">Tek bir öz bildirime dayanır. Yazışmanın seçilerek korunması, olumlu anlatım ve karşı tarafın sessizliği sonucu çarpıtabilir. İletişim, politika değişikliği anlamına gelmez.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sonraki kanıt: Neyi kontrol edeceğim?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atölye öncesi kayıtları, ikinci katılımcının anlatısını ve tarihli ortak taslağı karşılaştırırım. Çelişki bulursam iddiayı daraltırım; aynı kaynağın tekrarını bağımsız doğrulama saymam.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Şimdi tasarım kararları: Her satır bir araştırma tercihini açık eder. Veri yoksa sonuç uydurmak yerine hangi veriyi arayacağınızı yazın.</t>
+    <t xml:space="preserve">Ek kanıt: Doğrulanacak hususlar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atölye öncesi kayıtlar, ikinci katılımcının anlatısı ve tarihli ortak taslak karşılaştırılır. Çelişki varsa iddia daraltılır. Aynı kaynağın tekrarı bağımsız doğrulama sayılmaz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasarım kararları: Her satır bir araştırma tercihini açıklar. Veri bulunmuyorsa gerekli kanıtı belirtiniz ve sonuç iddiasını sınırlayınız.</t>
   </si>
   <si>
     <t xml:space="preserve">Tasarım kararı</t>
   </si>
   <si>
-    <t xml:space="preserve">Örnekte nasıl uygulanır?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benim araştırma planım</t>
+    <t xml:space="preserve">Örnekteki uygulama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Araştırma planı</t>
   </si>
   <si>
     <t xml:space="preserve">Araştırma sorusu</t>
@@ -779,19 +776,19 @@
     <t xml:space="preserve">İnceleme birimi</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir öğretmen çifti ve onun ortak çalışma süreci. Kişi, etkinlik ve ülke düzeyindeki iddiaları birbirine karıştırmam.</t>
+    <t xml:space="preserve">Bir öğretmen çifti ve ortak çalışma süreci. Kişi, etkinlik ve ülke düzeyindeki iddialar analitik olarak ayrı tutulur.</t>
   </si>
   <si>
     <t xml:space="preserve">Zaman ve kapsam</t>
   </si>
   <si>
-    <t xml:space="preserve">Varsayımsal plan: atölyeden önceki ve sonraki üç ay. Bu sınırın dışındaki olayları ancak gerekçesini belirterek eklerim.</t>
+    <t xml:space="preserve">Varsayımsal plan: atölyeden önceki ve sonraki üç ay. Bu kapsamın dışındaki olaylar yalnızca açık bir gerekçeyle incelemeye eklenir.</t>
   </si>
   <si>
     <t xml:space="preserve">Beklenen mekanizma</t>
   </si>
   <si>
-    <t xml:space="preserve">Atölyede temas kurulması, ortak bir konu seçilmesi ve birlikte taslak hazırlanması. Her adım için ayrı bir iz ararım.</t>
+    <t xml:space="preserve">Atölyede temas kurulması, ortak bir konu seçilmesi ve birlikte taslak hazırlanması. Her aşama için ayrı bir gözlenebilir iz aranır.</t>
   </si>
   <si>
     <t xml:space="preserve">Gösterge ve tanımı</t>
@@ -803,28 +800,28 @@
     <t xml:space="preserve">Vaka seçimi</t>
   </si>
   <si>
-    <t xml:space="preserve">Yalnız başarı anlatılarını seçmem. Devam etmeyen temasları da arar, hangi kişilerin veya belgelerin neden dışarıda kaldığını kaydederim.</t>
+    <t xml:space="preserve">Vaka seçimi başarı anlatılarıyla sınırlanmaz. Sürmeyen temaslar da araştırılır. Kişi veya belgelerin dışarıda bırakılma nedenleri kaydedilir.</t>
   </si>
   <si>
     <t xml:space="preserve">Karşılaştırma ve karşı olgu</t>
   </si>
   <si>
-    <t xml:space="preserve">Atölye öncesindeki işbirliğini ve uygun benzer katılmayan kişileri araştırırım. Grupların başlangıçta farklı olabileceğini açıklarım; benzerliği otomatik varsaymam.</t>
+    <t xml:space="preserve">Atölye öncesindeki işbirliği ve karşılaştırmaya uygun katılmayan kişiler araştırılır. Grupların başlangıç farklılıkları açıklanır. Karşılaştırılabilirlik varsayılmaz.</t>
   </si>
   <si>
     <t xml:space="preserve">Etik ve veri yönetimi</t>
   </si>
   <si>
-    <t xml:space="preserve">Gönüllü katılım, uygun izin, kişisel bilgilerin azaltılması ve güvenli saklama planı kurarım. Öğrenci verilerini bu çalışma kitabına kopyalamam.</t>
+    <t xml:space="preserve">Gönüllü katılım, uygun izin, kişisel verilerin en aza indirilmesi ve güvenli saklama planlanır. Öğrenci verileri bu çalışma kitabına aktarılmaz.</t>
   </si>
   <si>
     <t xml:space="preserve">Kaynak gösterme ve denetim izi</t>
   </si>
   <si>
-    <t xml:space="preserve">Yazar, tarih, başlık, koleksiyon veya yayın, kayıt/sayfa ve erişim bilgisini kaydederim. Çeviri, eksik belge ve değişen yorum için kısa bir işlem günlüğü tutarım.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teslim öncesi: İddia, gözlem, yorum ve sınır ayrı mı? En güçlü rakip açıklamayı sınamak için hangi kanıt gerekiyor?</t>
+    <t xml:space="preserve">Yazar, tarih, başlık, koleksiyon veya yayın, kayıt/sayfa ve erişim bilgisi kaydedilir. Çeviri, eksik belge ve değişen yorum için kısa bir işlem günlüğü tutulur.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teslim öncesi değerlendirme: İddia, gözlem, yorum ve sınırlılık ayrılmış mıdır? En güçlü rakip açıklamayı sınamak için hangi kanıt gereklidir?</t>
   </si>
   <si>
     <t xml:space="preserve">Ders dayanağı: 6. hafta değişimler, 14. hafta kanıt ve değerlendirme. Kurmaca örnek herhangi bir tarihsel sonuca kanıt oluşturmaz.</t>
@@ -1487,11 +1484,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="73527653"/>
-        <c:axId val="48016607"/>
+        <c:axId val="5306518"/>
+        <c:axId val="26188151"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="73527653"/>
+        <c:axId val="5306518"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1536,7 +1533,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48016607"/>
+        <c:crossAx val="26188151"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1544,7 +1541,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="48016607"/>
+        <c:axId val="26188151"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1589,7 +1586,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73527653"/>
+        <c:crossAx val="5306518"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2925,29 +2922,29 @@
         <v>89</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="H17" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>95</v>
       </c>
       <c r="I17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="74" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -2960,7 +2957,7 @@
     <row r="19" customFormat="false" ht="74" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -2973,7 +2970,7 @@
     <row r="20" customFormat="false" ht="74" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
@@ -2986,7 +2983,7 @@
     <row r="21" customFormat="false" ht="74" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
@@ -3010,7 +3007,7 @@
     <row r="23" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -3034,7 +3031,7 @@
     <row r="25" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -3109,7 +3106,7 @@
     <row r="2" customFormat="false" ht="31" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3133,7 +3130,7 @@
     <row r="4" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -3146,7 +3143,7 @@
     <row r="5" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -3159,7 +3156,7 @@
     <row r="6" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -3172,7 +3169,7 @@
     <row r="7" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -3185,7 +3182,7 @@
     <row r="8" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -3198,32 +3195,32 @@
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>114</v>
       </c>
       <c r="I9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="29" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>1000</v>
@@ -3249,7 +3246,7 @@
     <row r="11" customFormat="false" ht="29" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C11" s="18" t="n">
         <v>1000</v>
@@ -3286,7 +3283,7 @@
     <row r="13" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -3310,25 +3307,25 @@
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="G15" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="H15" s="4" t="s">
         <v>122</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="I15" s="1"/>
     </row>
@@ -3355,7 +3352,7 @@
         <v>4</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H16" s="6" t="str">
         <f aca="false">IF(H10&lt;&gt;"Hazır",H10,"Destek değişimi: "&amp;TEXT(F16,"0.0")&amp;" yüzde puan. Nedeni henüz bilinmiyor.")</f>
@@ -3386,7 +3383,7 @@
         <v>15</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H17" s="14" t="str">
         <f aca="false">IF(H11&lt;&gt;"Hazır",H11,"Destek değişimi: "&amp;TEXT(F17,"0.0")&amp;" yüzde puan. Nedeni henüz bilinmiyor.")</f>
@@ -3408,7 +3405,7 @@
     <row r="19" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -3421,7 +3418,7 @@
     <row r="20" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -3599,7 +3596,7 @@
     <row r="36" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1"/>
       <c r="B36" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -3612,7 +3609,7 @@
     <row r="37" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1"/>
       <c r="B37" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -3625,7 +3622,7 @@
     <row r="38" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1"/>
       <c r="B38" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
@@ -3638,7 +3635,7 @@
     <row r="39" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1"/>
       <c r="B39" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
@@ -3662,32 +3659,32 @@
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1"/>
       <c r="B41" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="D41" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="E41" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="E41" s="4" t="s">
+      <c r="F41" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="G41" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="H41" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>138</v>
       </c>
       <c r="I41" s="1"/>
     </row>
     <row r="42" customFormat="false" ht="88" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1"/>
       <c r="B42" s="23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C42" s="24"/>
       <c r="D42" s="24"/>
@@ -3722,7 +3719,7 @@
     <row r="45" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1"/>
       <c r="B45" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
@@ -3735,7 +3732,7 @@
     <row r="46" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1"/>
       <c r="B46" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -3759,7 +3756,7 @@
     <row r="48" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1"/>
       <c r="B48" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
@@ -3871,7 +3868,7 @@
     <row r="2" customFormat="false" ht="31" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3891,7 +3888,7 @@
     <row r="4" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -3911,16 +3908,16 @@
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>148</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -3928,16 +3925,16 @@
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>151</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -3945,16 +3942,16 @@
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="D8" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="E8" s="10" t="s">
         <v>155</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>156</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -3962,16 +3959,16 @@
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -3979,16 +3976,16 @@
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="D10" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="E10" s="10" t="s">
         <v>163</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>164</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
@@ -3996,16 +3993,16 @@
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="D11" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>168</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
@@ -4013,16 +4010,16 @@
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="10" t="s">
         <v>171</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>172</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -4030,16 +4027,16 @@
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="10" t="s">
         <v>175</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>176</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -4047,16 +4044,16 @@
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="E14" s="10" t="s">
         <v>179</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>180</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -4064,16 +4061,16 @@
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="E15" s="10" t="s">
         <v>183</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>184</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -4081,16 +4078,16 @@
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
       <c r="B16" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="E16" s="10" t="s">
         <v>187</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>188</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -4098,16 +4095,16 @@
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
       <c r="B17" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="D17" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="E17" s="10" t="s">
         <v>191</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>192</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -4115,16 +4112,16 @@
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="E18" s="10" t="s">
         <v>195</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>196</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -4132,16 +4129,16 @@
     <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="E19" s="10" t="s">
         <v>199</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>200</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -4149,16 +4146,16 @@
     <row r="20" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="E20" s="10" t="s">
         <v>203</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>204</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -4166,16 +4163,16 @@
     <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="D21" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="E21" s="10" t="s">
         <v>207</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>208</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
@@ -4183,16 +4180,16 @@
     <row r="22" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="D22" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="E22" s="10" t="s">
         <v>211</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>212</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -4200,16 +4197,16 @@
     <row r="23" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="D23" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="E23" s="10" t="s">
         <v>215</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>216</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -4217,16 +4214,16 @@
     <row r="24" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
       <c r="B24" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>217</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="D24" s="14" t="s">
         <v>218</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="E24" s="14" t="s">
         <v>219</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>220</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -4252,7 +4249,7 @@
     <row r="27" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -4338,7 +4335,7 @@
     <row r="2" customFormat="false" ht="31" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4354,7 +4351,7 @@
     <row r="4" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -4363,7 +4360,7 @@
     <row r="5" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -4372,7 +4369,7 @@
     <row r="6" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -4381,7 +4378,7 @@
     <row r="7" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -4397,23 +4394,23 @@
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>228</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>229</v>
       </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>230</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>231</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="1"/>
@@ -4421,10 +4418,10 @@
     <row r="11" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>232</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>233</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="1"/>
@@ -4432,10 +4429,10 @@
     <row r="12" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>234</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>235</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="1"/>
@@ -4443,10 +4440,10 @@
     <row r="13" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>236</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>237</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="1"/>
@@ -4454,10 +4451,10 @@
     <row r="14" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>238</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>239</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="1"/>
@@ -4465,10 +4462,10 @@
     <row r="15" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>240</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>241</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="1"/>
@@ -4476,10 +4473,10 @@
     <row r="16" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
       <c r="B16" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="C16" s="14" t="s">
         <v>242</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="1"/>
@@ -4494,7 +4491,7 @@
     <row r="18" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -4510,23 +4507,23 @@
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>247</v>
       </c>
       <c r="E20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>248</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>249</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="1"/>
@@ -4534,10 +4531,10 @@
     <row r="22" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>250</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>251</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="1"/>
@@ -4545,10 +4542,10 @@
     <row r="23" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>252</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>253</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="1"/>
@@ -4556,10 +4553,10 @@
     <row r="24" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
       <c r="B24" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>254</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>255</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="1"/>
@@ -4567,10 +4564,10 @@
     <row r="25" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
       <c r="B25" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>256</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>257</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="1"/>
@@ -4578,10 +4575,10 @@
     <row r="26" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
       <c r="B26" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>258</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>259</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="1"/>
@@ -4589,10 +4586,10 @@
     <row r="27" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>260</v>
-      </c>
-      <c r="C27" s="10" t="s">
-        <v>261</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="1"/>
@@ -4600,10 +4597,10 @@
     <row r="28" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
       <c r="B28" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>262</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>263</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="1"/>
@@ -4611,10 +4608,10 @@
     <row r="29" customFormat="false" ht="76" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1"/>
       <c r="B29" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>264</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>265</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="1"/>
@@ -4629,7 +4626,7 @@
     <row r="31" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -4638,7 +4635,7 @@
     <row r="32" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1"/>
       <c r="B32" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>

</xml_diff>